<commit_message>
Excel parser funcionando, aberto implementações
</commit_message>
<xml_diff>
--- a/modelos/MODELO.xlsx
+++ b/modelos/MODELO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Trabalho Matheus\FRIGORIFICO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{78786F5B-07C8-43FE-B9E5-8AD46AE938B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{981BF1C3-8770-4679-AEAE-75D5034696F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{22414FF8-6C4D-4CCC-970D-B9C2150EA6EE}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>LOJA</t>
   </si>
@@ -60,7 +60,19 @@
     <t xml:space="preserve">FATURADO POR </t>
   </si>
   <si>
-    <t>COMISSÃO</t>
+    <t>FILÉ DE COSTELA (ANCHO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> SABOR DO CHURRASCO</t>
+  </si>
+  <si>
+    <t>7 14 21</t>
+  </si>
+  <si>
+    <t>FRIGORÍFICO  VISCONDE</t>
+  </si>
+  <si>
+    <t>COMISSAO</t>
   </si>
 </sst>
 </file>
@@ -108,7 +120,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -121,14 +133,8 @@
         <bgColor rgb="FF666699"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -149,6 +155,32 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -164,9 +196,6 @@
     <xf numFmtId="4" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -182,11 +211,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -194,7 +226,21 @@
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -570,36 +616,54 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="3" t="s">
-        <v>11</v>
+      <c r="L1" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="5">
+      <c r="A2" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="3">
+        <v>25</v>
+      </c>
+      <c r="D2" s="3">
+        <v>1</v>
+      </c>
+      <c r="E2" s="4">
         <f>C2*D2</f>
-        <v>0</v>
-      </c>
-      <c r="F2" s="6"/>
-      <c r="G2" s="7">
+        <v>25</v>
+      </c>
+      <c r="F2" s="5">
+        <v>36</v>
+      </c>
+      <c r="G2" s="6">
         <f>(F2*C2)*D2</f>
-        <v>0</v>
-      </c>
-      <c r="H2" s="10"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8">
+        <v>900</v>
+      </c>
+      <c r="H2" s="8">
+        <v>46237</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="9">
+        <v>46240</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="L2" s="7">
         <f>G2*0.01</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2">
-    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>